<commit_message>
Producción: Sistema verificado, umbral de ballenas restablecido a 80k
</commit_message>
<xml_diff>
--- a/Dashboard_Trading.xlsx
+++ b/Dashboard_Trading.xlsx
@@ -443,14 +443,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CCL: $1426.88</t>
+          <t>CCL: $1430.25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="D4" t="inlineStr">
         <is>
-          <t>Local: $6650.00</t>
+          <t>Local: $6700.00</t>
         </is>
       </c>
     </row>

</xml_diff>